<commit_message>
Thinking in Java C1
</commit_message>
<xml_diff>
--- a/doc/Java.xlsx
+++ b/doc/Java.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hades/Documents/GitHub/JavaAboutDemos/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2DB498E-0A2B-0A4C-8687-734EA25CEFE2}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9E9C86-C8C8-2748-9360-1DD33BEB60B2}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{7C69AD57-AE32-C847-879F-875651E96C78}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>Usage</t>
   </si>
@@ -194,12 +194,21 @@
   <si>
     <t>图形化界面</t>
   </si>
+  <si>
+    <t>新东西</t>
+  </si>
+  <si>
+    <t>其他语言里中类似基本概念</t>
+  </si>
+  <si>
+    <t>封装</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -226,8 +235,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -237,6 +252,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FA00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -282,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -304,12 +331,21 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF00FA00"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1158,31 +1194,37 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6601D41D-AD5A-BE45-B683-D4A75B94E650}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
+      <c r="C1" s="14" t="s">
+        <v>47</v>
+      </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
       <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="G1" s="14" t="s">
+        <v>49</v>
+      </c>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:10">
       <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
+      <c r="C2" s="11" t="s">
+        <v>35</v>
+      </c>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="9" t="s">
-        <v>49</v>
+      <c r="H2" s="12" t="s">
+        <v>52</v>
       </c>
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
@@ -1192,15 +1234,12 @@
         <v>21</v>
       </c>
       <c r="B3" s="9"/>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="11" t="s">
         <v>32</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="11" t="s">
         <v>34</v>
       </c>
       <c r="H3" s="9"/>
@@ -1209,15 +1248,12 @@
     </row>
     <row r="4" spans="1:10">
       <c r="B4" s="9"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="11" t="s">
         <v>30</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>47</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="11" t="s">
         <v>36</v>
       </c>
       <c r="H4" s="9"/>
@@ -1226,13 +1262,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="B5" s="9"/>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
       <c r="F5" s="9"/>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="11" t="s">
         <v>40</v>
       </c>
       <c r="H5" s="9"/>
@@ -1241,13 +1277,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="B6" s="9"/>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="11" t="s">
         <v>43</v>
       </c>
       <c r="H6" s="9"/>
@@ -1256,13 +1292,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="B7" s="9"/>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="11" t="s">
         <v>26</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="11" t="s">
         <v>48</v>
       </c>
       <c r="H7" s="9"/>
@@ -1282,13 +1318,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="B9" s="9"/>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="11" t="s">
         <v>37</v>
       </c>
       <c r="H9" s="9"/>
@@ -1297,13 +1333,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="B10" s="9"/>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="11" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="11" t="s">
         <v>39</v>
       </c>
       <c r="H10" s="9"/>
@@ -1315,13 +1351,13 @@
         <v>22</v>
       </c>
       <c r="B11" s="9"/>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="11" t="s">
         <v>31</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="11" t="s">
         <v>44</v>
       </c>
       <c r="H11" s="9"/>
@@ -1330,13 +1366,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="B12" s="9"/>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="14" t="s">
         <v>45</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="11" t="s">
         <v>38</v>
       </c>
       <c r="H12" s="9"/>
@@ -1349,7 +1385,7 @@
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="11" t="s">
         <v>46</v>
       </c>
       <c r="H13" s="9"/>
@@ -1418,6 +1454,16 @@
         <v>42</v>
       </c>
     </row>
+    <row r="22" spans="2:10">
+      <c r="B22" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10">
+      <c r="B23" s="13" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>